<commit_message>
Add that judge model can't be same as base model
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>Llama-2-7b-chat-hf</t>
   </si>
@@ -62,9 +62,6 @@
   </si>
   <si>
     <t>ASR: 0.8197 | V1: 61</t>
-  </si>
-  <si>
-    <t>ASR: 0.4359 | V1: 39</t>
   </si>
   <si>
     <t>ASR: 0.4812 | V1: 133</t>
@@ -492,10 +489,10 @@
         <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -509,13 +506,13 @@
         <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -525,20 +522,17 @@
       <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
       <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" t="s">
-        <v>19</v>
-      </c>
       <c r="G4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Archive result files with same judges as base model
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>Llama-2-7b-chat-hf</t>
   </si>
@@ -46,49 +46,43 @@
     <t>Llama-3.3-70B-Instruct</t>
   </si>
   <si>
+    <t>ASR: 0.2308 | V1: 52</t>
+  </si>
+  <si>
     <t>ASR: 0.2016 | V1: 129</t>
   </si>
   <si>
+    <t>ASR: 0.6098 | V1: 41</t>
+  </si>
+  <si>
     <t>ASR: 0.8148 | V1: 81</t>
   </si>
   <si>
-    <t>ASR: 0.8500 | V1: 40</t>
-  </si>
-  <si>
-    <t>ASR: 0.6098 | V1: 41</t>
-  </si>
-  <si>
     <t>ASR: 0.4130 | V1: 92</t>
   </si>
   <si>
     <t>ASR: 0.8197 | V1: 61</t>
   </si>
   <si>
+    <t>ASR: 0.2889 | V1: 90</t>
+  </si>
+  <si>
     <t>ASR: 0.4812 | V1: 133</t>
   </si>
   <si>
-    <t>ASR: 0.2889 | V1: 90</t>
-  </si>
-  <si>
     <t>ASR: 0.6176 | V1: 34</t>
   </si>
   <si>
-    <t>ASR: 0.7797 | V1: 118</t>
+    <t>ASR: 0.6724 | V1: 58</t>
   </si>
   <si>
     <t>ASR: 0.7091 | V1: 110</t>
   </si>
   <si>
-    <t>ASR: 0.6724 | V1: 58</t>
+    <t>ASR: 0.7500 | V1: 36</t>
   </si>
   <si>
     <t>ASR: 0.9483 | V1: 58</t>
-  </si>
-  <si>
-    <t>ASR: 0.9828 | V1: 58</t>
-  </si>
-  <si>
-    <t>ASR: 0.7500 | V1: 36</t>
   </si>
 </sst>
 </file>
@@ -477,62 +471,56 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>14</v>
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
       </c>
       <c r="G2" t="s">
         <v>19</v>
       </c>
       <c r="H2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
       </c>
       <c r="E4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" t="s">
-        <v>18</v>
-      </c>
       <c r="G4" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restore accidentally removed files
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>Llama-2-7b-chat-hf</t>
   </si>
@@ -83,6 +83,9 @@
   </si>
   <si>
     <t>ASR: 0.9483 | V1: 58</t>
+  </si>
+  <si>
+    <t>ASR: 0.9828 | V1: 58</t>
   </si>
 </sst>
 </file>
@@ -522,6 +525,9 @@
       <c r="G4" t="s">
         <v>20</v>
       </c>
+      <c r="H4" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add phi results, improve overview table
</commit_message>
<xml_diff>
--- a/overview.xlsx
+++ b/overview.xlsx
@@ -7,14 +7,14 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="ASR Overview" sheetId="1" r:id="rId1"/>
+    <sheet name="ASR-Overview" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
   <si>
     <t>Llama-2-7b-chat-hf</t>
   </si>
@@ -40,52 +40,89 @@
     <t>Judge Model</t>
   </si>
   <si>
+    <t>Llama-3.3-70B-Instruct</t>
+  </si>
+  <si>
     <t>Qwen2.5-72B-Instruct</t>
   </si>
   <si>
-    <t>Llama-3.3-70B-Instruct</t>
-  </si>
-  <si>
-    <t>ASR: 0.2308 | V1: 52</t>
-  </si>
-  <si>
-    <t>ASR: 0.2016 | V1: 129</t>
-  </si>
-  <si>
-    <t>ASR: 0.6098 | V1: 41</t>
-  </si>
-  <si>
-    <t>ASR: 0.8148 | V1: 81</t>
-  </si>
-  <si>
-    <t>ASR: 0.4130 | V1: 92</t>
-  </si>
-  <si>
-    <t>ASR: 0.8197 | V1: 61</t>
-  </si>
-  <si>
-    <t>ASR: 0.2889 | V1: 90</t>
-  </si>
-  <si>
-    <t>ASR: 0.4812 | V1: 133</t>
-  </si>
-  <si>
-    <t>ASR: 0.6176 | V1: 34</t>
-  </si>
-  <si>
-    <t>ASR: 0.6724 | V1: 58</t>
-  </si>
-  <si>
-    <t>ASR: 0.7091 | V1: 110</t>
-  </si>
-  <si>
-    <t>ASR: 0.7500 | V1: 36</t>
-  </si>
-  <si>
-    <t>ASR: 0.9483 | V1: 58</t>
-  </si>
-  <si>
-    <t>ASR: 0.9828 | V1: 58</t>
+    <t>phi-4</t>
+  </si>
+  <si>
+    <t>ASR: 0.20
+V1: 129 V2: 2 Vties: 11</t>
+  </si>
+  <si>
+    <t>ASR: 0.57
+V1: 128 V2: 4 Vties: 3</t>
+  </si>
+  <si>
+    <t>ASR: 0.23
+V1: 52 V2: 10 Vties: 76</t>
+  </si>
+  <si>
+    <t>ASR: 0.81
+V1: 81 V2: 19 Vties: 42</t>
+  </si>
+  <si>
+    <t>ASR: 0.78
+V1: 81 V2: 25 Vties: 7</t>
+  </si>
+  <si>
+    <t>ASR: 0.61
+V1: 41 V2: 10 Vties: 89</t>
+  </si>
+  <si>
+    <t>ASR: 0.82
+V1: 61 V2: 35 Vties: 46</t>
+  </si>
+  <si>
+    <t>ASR: 0.41
+V1: 92 V2: 16 Vties: 34</t>
+  </si>
+  <si>
+    <t>ASR: 0.77
+V1: 88 V2: 20 Vties: 12</t>
+  </si>
+  <si>
+    <t>ASR: 0.48
+V1: 133 V2: 3 Vties: 6</t>
+  </si>
+  <si>
+    <t>ASR: 0.22
+V1: 138 V2: 0 Vties: 4</t>
+  </si>
+  <si>
+    <t>ASR: 0.29
+V1: 90 V2: 1 Vties: 50</t>
+  </si>
+  <si>
+    <t>ASR: 0.82
+V1: 49 V2: 53 Vties: 16</t>
+  </si>
+  <si>
+    <t>ASR: 0.62
+V1: 34 V2: 15 Vties: 92</t>
+  </si>
+  <si>
+    <t>ASR: 0.71
+V1: 110 V2: 12 Vties: 20</t>
+  </si>
+  <si>
+    <t>ASR: 0.67
+V1: 58 V2: 11 Vties: 72</t>
+  </si>
+  <si>
+    <t>ASR: 0.98
+V1: 58 V2: 29 Vties: 55</t>
+  </si>
+  <si>
+    <t>ASR: 0.95
+V1: 58 V2: 12 Vties: 72</t>
+  </si>
+  <si>
+    <t>ASR: 0.75
+V1: 36 V2: 7 Vties: 99</t>
   </si>
 </sst>
 </file>
@@ -144,8 +181,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -443,90 +483,113 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="8" width="20.7109375" style="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
+      <c r="A2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="A3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="D3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="A4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="D4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>